<commit_message>
updating log for final FA23 deployments
</commit_message>
<xml_diff>
--- a/TFO_Drifter_deployment_log.xlsx
+++ b/TFO_Drifter_deployment_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/sio_research/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACA79063-C8B8-F54A-A910-8441FD26CC4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0205BF3D-FBD2-4744-97E0-4FEDFB7DBAFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="57">
   <si>
     <t>Deployment</t>
   </si>
@@ -205,6 +205,12 @@
   <si>
     <t xml:space="preserve">Time Zone Offset </t>
   </si>
+  <si>
+    <t>Drifter 6 and 4 deployed in close proximity. Drifter 6 deployed with DURIP payload hanging below. Difficulty offloading data, system freezing</t>
+  </si>
+  <si>
+    <t>Drifter 6 and 4 deployed in close proximity. Channel 9 contains loud contamination (not an acoustic channel)</t>
+  </si>
 </sst>
 </file>
 
@@ -215,7 +221,7 @@
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\Thh:mm:ss"/>
     <numFmt numFmtId="166" formatCode="hh:mm"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -269,6 +275,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -290,7 +303,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -313,12 +326,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -348,7 +374,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -427,8 +452,49 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="21" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="22" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="22" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -672,153 +738,153 @@
     <col min="28" max="16384" width="14.5" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="41" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:27" s="40" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="35" t="s">
+      <c r="E1" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="36" t="s">
+      <c r="F1" s="35" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="34" t="s">
+      <c r="G1" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="H1" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="35" t="s">
+      <c r="I1" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="J1" s="39" t="s">
+      <c r="J1" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="34" t="s">
+      <c r="K1" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="34" t="s">
+      <c r="L1" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="M1" s="34" t="s">
+      <c r="M1" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="N1" s="34" t="s">
+      <c r="N1" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="37" t="s">
+      <c r="O1" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="P1" s="37" t="s">
+      <c r="P1" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="Q1" s="38" t="s">
+      <c r="Q1" s="37" t="s">
         <v>10</v>
       </c>
-      <c r="R1" s="34" t="s">
+      <c r="R1" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="S1" s="34" t="s">
+      <c r="S1" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="T1" s="38" t="s">
+      <c r="T1" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="U1" s="34" t="s">
+      <c r="U1" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="V1" s="34" t="s">
+      <c r="V1" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="W1" s="40" t="s">
+      <c r="W1" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="X1" s="40" t="s">
+      <c r="X1" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="Y1" s="34" t="s">
+      <c r="Y1" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="Z1" s="34" t="s">
+      <c r="Z1" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="AA1" s="34" t="s">
+      <c r="AA1" s="33" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:27" s="21" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="14">
+    <row r="2" spans="1:27" s="20" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="13">
         <v>1</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="14">
+      <c r="C2" s="13">
         <v>4</v>
       </c>
-      <c r="D2" s="14">
+      <c r="D2" s="13">
         <v>1</v>
       </c>
-      <c r="E2" s="15">
+      <c r="E2" s="14">
         <v>44818</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="15">
         <v>0.55138888888888882</v>
       </c>
-      <c r="G2" s="14">
+      <c r="G2" s="13">
         <v>39.865239000000003</v>
       </c>
-      <c r="H2" s="14">
+      <c r="H2" s="13">
         <v>-70.443644000000006</v>
       </c>
-      <c r="I2" s="15">
+      <c r="I2" s="14">
         <v>44818</v>
       </c>
-      <c r="J2" s="19">
+      <c r="J2" s="18">
         <v>0.66666666666666663</v>
       </c>
-      <c r="K2" s="14">
+      <c r="K2" s="13">
         <v>39.869919000000003</v>
       </c>
-      <c r="L2" s="14">
+      <c r="L2" s="13">
         <v>-70.432182999999995</v>
       </c>
-      <c r="M2" s="14">
+      <c r="M2" s="13">
         <v>1</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="N2" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="O2" s="17">
+      <c r="O2" s="16">
         <v>300434066482170</v>
       </c>
-      <c r="P2" s="17" t="s">
+      <c r="P2" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="Q2" s="18"/>
-      <c r="R2" s="14"/>
-      <c r="S2" s="14"/>
-      <c r="T2" s="18"/>
-      <c r="U2" s="14"/>
-      <c r="V2" s="14"/>
-      <c r="W2" s="20">
+      <c r="Q2" s="17"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="13"/>
+      <c r="T2" s="17"/>
+      <c r="U2" s="13"/>
+      <c r="V2" s="13"/>
+      <c r="W2" s="19">
         <v>0.43124999999999997</v>
       </c>
-      <c r="X2" s="20">
+      <c r="X2" s="19">
         <v>0.45208333333333334</v>
       </c>
-      <c r="Y2" s="14"/>
-      <c r="Z2" s="14"/>
-      <c r="AA2" s="14" t="s">
+      <c r="Y2" s="13"/>
+      <c r="Z2" s="13"/>
+      <c r="AA2" s="13" t="s">
         <v>24</v>
       </c>
     </row>
@@ -901,78 +967,78 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:27" s="21" customFormat="1" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="14">
+    <row r="4" spans="1:27" s="20" customFormat="1" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="13">
         <v>3</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="14">
+      <c r="C4" s="13">
         <v>4</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4" s="13">
         <v>1</v>
       </c>
-      <c r="E4" s="15">
+      <c r="E4" s="14">
         <v>44822</v>
       </c>
-      <c r="F4" s="16"/>
-      <c r="G4" s="14">
+      <c r="F4" s="15"/>
+      <c r="G4" s="13">
         <v>38.944544999999998</v>
       </c>
-      <c r="H4" s="14">
+      <c r="H4" s="13">
         <v>-63.757482000000003</v>
       </c>
-      <c r="I4" s="15"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="14">
+      <c r="I4" s="14"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="13">
         <v>38.974831000000002</v>
       </c>
-      <c r="L4" s="14">
+      <c r="L4" s="13">
         <v>-63.683495000000001</v>
       </c>
-      <c r="M4" s="14">
+      <c r="M4" s="13">
         <v>1</v>
       </c>
-      <c r="N4" s="14" t="s">
+      <c r="N4" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="O4" s="17">
+      <c r="O4" s="16">
         <v>300434066482170</v>
       </c>
-      <c r="P4" s="17" t="s">
+      <c r="P4" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="Q4" s="18">
+      <c r="Q4" s="17">
         <v>44822.083333333336</v>
       </c>
-      <c r="R4" s="14">
+      <c r="R4" s="13">
         <v>38.941955</v>
       </c>
-      <c r="S4" s="14">
+      <c r="S4" s="13">
         <v>-63.756053000000001</v>
       </c>
-      <c r="T4" s="18">
+      <c r="T4" s="17">
         <v>44822.465277777781</v>
       </c>
-      <c r="U4" s="14">
+      <c r="U4" s="13">
         <v>38.973402999999998</v>
       </c>
-      <c r="V4" s="14">
+      <c r="V4" s="13">
         <v>-63.696891999999998</v>
       </c>
-      <c r="W4" s="20">
+      <c r="W4" s="19">
         <v>0.41597222222222219</v>
       </c>
-      <c r="X4" s="20">
+      <c r="X4" s="19">
         <v>0.92986111111111114</v>
       </c>
-      <c r="Y4" s="14">
+      <c r="Y4" s="13">
         <v>250</v>
       </c>
-      <c r="Z4" s="14"/>
-      <c r="AA4" s="14" t="s">
+      <c r="Z4" s="13"/>
+      <c r="AA4" s="13" t="s">
         <v>26</v>
       </c>
     </row>
@@ -1049,78 +1115,78 @@
       <c r="Z5" s="1"/>
       <c r="AA5" s="1"/>
     </row>
-    <row r="6" spans="1:27" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="22">
+    <row r="6" spans="1:27" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="21">
         <v>5</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="22">
+      <c r="C6" s="21">
         <v>4</v>
       </c>
-      <c r="D6" s="22">
+      <c r="D6" s="21">
         <v>1</v>
       </c>
-      <c r="E6" s="23">
+      <c r="E6" s="22">
         <v>44823</v>
       </c>
-      <c r="F6" s="24"/>
-      <c r="G6" s="22">
+      <c r="F6" s="23"/>
+      <c r="G6" s="21">
         <v>38.885973999999997</v>
       </c>
-      <c r="H6" s="22">
+      <c r="H6" s="21">
         <v>-64.015152</v>
       </c>
-      <c r="I6" s="23"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="22">
+      <c r="I6" s="22"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="21">
         <v>38.879128999999999</v>
       </c>
-      <c r="L6" s="22">
+      <c r="L6" s="21">
         <v>-63.895172000000002</v>
       </c>
-      <c r="M6" s="22">
+      <c r="M6" s="21">
         <v>1</v>
       </c>
-      <c r="N6" s="22" t="s">
+      <c r="N6" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="O6" s="25">
+      <c r="O6" s="24">
         <v>300434066482170</v>
       </c>
-      <c r="P6" s="25" t="s">
+      <c r="P6" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="Q6" s="26">
+      <c r="Q6" s="25">
         <v>44823.822916666664</v>
       </c>
-      <c r="R6" s="22">
+      <c r="R6" s="21">
         <v>38.886195999999998</v>
       </c>
-      <c r="S6" s="22">
+      <c r="S6" s="21">
         <v>-64.012355999999997</v>
       </c>
-      <c r="T6" s="26">
+      <c r="T6" s="25">
         <v>44824.329861111109</v>
       </c>
-      <c r="U6" s="22">
+      <c r="U6" s="21">
         <v>38.854120000000002</v>
       </c>
-      <c r="V6" s="22">
+      <c r="V6" s="21">
         <v>-63.966763999999998</v>
       </c>
-      <c r="W6" s="28">
+      <c r="W6" s="27">
         <v>0.41666666666666669</v>
       </c>
-      <c r="X6" s="28">
+      <c r="X6" s="27">
         <v>0.92847222222222225</v>
       </c>
-      <c r="Y6" s="22">
+      <c r="Y6" s="21">
         <v>400</v>
       </c>
-      <c r="Z6" s="22"/>
-      <c r="AA6" s="22" t="s">
+      <c r="Z6" s="21"/>
+      <c r="AA6" s="21" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1197,249 +1263,249 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:27" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="22">
+    <row r="8" spans="1:27" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="21">
         <v>7</v>
       </c>
-      <c r="B8" s="22"/>
-      <c r="C8" s="22">
+      <c r="B8" s="21"/>
+      <c r="C8" s="21">
         <v>4</v>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="21">
         <v>1</v>
       </c>
-      <c r="E8" s="23">
+      <c r="E8" s="22">
         <v>44983</v>
       </c>
-      <c r="F8" s="24"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-      <c r="I8" s="23"/>
-      <c r="J8" s="27"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="22"/>
-      <c r="M8" s="22">
+      <c r="F8" s="23"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="21"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="26"/>
+      <c r="K8" s="21"/>
+      <c r="L8" s="21"/>
+      <c r="M8" s="21">
         <v>1</v>
       </c>
-      <c r="N8" s="22" t="s">
+      <c r="N8" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="O8" s="25">
+      <c r="O8" s="24">
         <v>300434066480130</v>
       </c>
-      <c r="P8" s="25" t="s">
+      <c r="P8" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="Q8" s="26">
+      <c r="Q8" s="25">
         <v>44983.875324074077</v>
       </c>
-      <c r="R8" s="22">
+      <c r="R8" s="21">
         <v>32.910995</v>
       </c>
-      <c r="S8" s="22">
+      <c r="S8" s="21">
         <v>-117.74101400000001</v>
       </c>
-      <c r="T8" s="26">
+      <c r="T8" s="25">
         <v>44984.385752314818</v>
       </c>
-      <c r="U8" s="22">
+      <c r="U8" s="21">
         <v>32.911644000000003</v>
       </c>
-      <c r="V8" s="22">
+      <c r="V8" s="21">
         <v>-117.73635299999999</v>
       </c>
-      <c r="W8" s="28">
+      <c r="W8" s="27">
         <v>0.59861111111111109</v>
       </c>
-      <c r="X8" s="28">
+      <c r="X8" s="27">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="Y8" s="22"/>
-      <c r="Z8" s="22"/>
-      <c r="AA8" s="22"/>
-    </row>
-    <row r="9" spans="1:27" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="22">
+      <c r="Y8" s="21"/>
+      <c r="Z8" s="21"/>
+      <c r="AA8" s="21"/>
+    </row>
+    <row r="9" spans="1:27" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="21">
         <v>7</v>
       </c>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22">
+      <c r="B9" s="21"/>
+      <c r="C9" s="21">
         <v>4</v>
       </c>
-      <c r="D9" s="22">
+      <c r="D9" s="21">
         <v>2</v>
       </c>
-      <c r="E9" s="23">
+      <c r="E9" s="22">
         <v>44983</v>
       </c>
-      <c r="F9" s="24"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="27"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
-      <c r="M9" s="22">
+      <c r="F9" s="23"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="21"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="26"/>
+      <c r="K9" s="21"/>
+      <c r="L9" s="21"/>
+      <c r="M9" s="21">
         <v>1</v>
       </c>
-      <c r="N9" s="22" t="s">
+      <c r="N9" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="O9" s="25">
+      <c r="O9" s="24">
         <v>300434066480130</v>
       </c>
-      <c r="P9" s="25" t="s">
+      <c r="P9" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="Q9" s="26">
+      <c r="Q9" s="25">
         <v>44984.416990740741</v>
       </c>
-      <c r="R9" s="22">
+      <c r="R9" s="21">
         <v>32.908870999999998</v>
       </c>
-      <c r="S9" s="22">
+      <c r="S9" s="21">
         <v>-117.73746199999999</v>
       </c>
-      <c r="T9" s="26">
+      <c r="T9" s="25">
         <v>44984.896157407406</v>
       </c>
-      <c r="U9" s="22">
+      <c r="U9" s="21">
         <v>32.92512</v>
       </c>
-      <c r="V9" s="22">
+      <c r="V9" s="21">
         <v>-117.753174</v>
       </c>
-      <c r="W9" s="28">
+      <c r="W9" s="27">
         <v>0.59861111111111109</v>
       </c>
-      <c r="X9" s="28">
+      <c r="X9" s="27">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="Y9" s="22"/>
-      <c r="Z9" s="22"/>
-      <c r="AA9" s="22"/>
-    </row>
-    <row r="10" spans="1:27" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="22">
+      <c r="Y9" s="21"/>
+      <c r="Z9" s="21"/>
+      <c r="AA9" s="21"/>
+    </row>
+    <row r="10" spans="1:27" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="21">
         <v>7</v>
       </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22">
+      <c r="B10" s="21"/>
+      <c r="C10" s="21">
         <v>4</v>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="21">
         <v>3</v>
       </c>
-      <c r="E10" s="23">
+      <c r="E10" s="22">
         <v>44983</v>
       </c>
-      <c r="F10" s="24"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
-      <c r="M10" s="22">
+      <c r="F10" s="23"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="21"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
+      <c r="M10" s="21">
         <v>1</v>
       </c>
-      <c r="N10" s="22" t="s">
+      <c r="N10" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="O10" s="25">
+      <c r="O10" s="24">
         <v>300434066480130</v>
       </c>
-      <c r="P10" s="25" t="s">
+      <c r="P10" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="Q10" s="26">
+      <c r="Q10" s="25">
         <v>44984.896157407406</v>
       </c>
-      <c r="R10" s="22">
+      <c r="R10" s="21">
         <v>32.92512</v>
       </c>
-      <c r="S10" s="22">
+      <c r="S10" s="21">
         <v>-117.753174</v>
       </c>
-      <c r="T10" s="26">
+      <c r="T10" s="25">
         <v>44985.399629629632</v>
       </c>
-      <c r="U10" s="22">
+      <c r="U10" s="21">
         <v>32.922975999999998</v>
       </c>
-      <c r="V10" s="22">
+      <c r="V10" s="21">
         <v>-117.769451</v>
       </c>
-      <c r="W10" s="28">
+      <c r="W10" s="27">
         <v>0.59861111111111109</v>
       </c>
-      <c r="X10" s="28">
+      <c r="X10" s="27">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="Y10" s="22"/>
-      <c r="Z10" s="22"/>
-      <c r="AA10" s="22"/>
-    </row>
-    <row r="11" spans="1:27" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="22">
+      <c r="Y10" s="21"/>
+      <c r="Z10" s="21"/>
+      <c r="AA10" s="21"/>
+    </row>
+    <row r="11" spans="1:27" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="21">
         <v>7</v>
       </c>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22">
+      <c r="B11" s="21"/>
+      <c r="C11" s="21">
         <v>4</v>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="21">
         <v>4</v>
       </c>
-      <c r="E11" s="23">
+      <c r="E11" s="22">
         <v>44983</v>
       </c>
-      <c r="F11" s="24"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
-      <c r="I11" s="23"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="22"/>
-      <c r="L11" s="22"/>
-      <c r="M11" s="22">
+      <c r="F11" s="23"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="22"/>
+      <c r="J11" s="26"/>
+      <c r="K11" s="21"/>
+      <c r="L11" s="21"/>
+      <c r="M11" s="21">
         <v>1</v>
       </c>
-      <c r="N11" s="22" t="s">
+      <c r="N11" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="O11" s="25">
+      <c r="O11" s="24">
         <v>300434066480130</v>
       </c>
-      <c r="P11" s="25" t="s">
+      <c r="P11" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="Q11" s="26">
+      <c r="Q11" s="25">
         <v>44985.403113425928</v>
       </c>
-      <c r="R11" s="22">
+      <c r="R11" s="21">
         <v>32.922437000000002</v>
       </c>
-      <c r="S11" s="22">
+      <c r="S11" s="21">
         <v>-117.76988799999999</v>
       </c>
-      <c r="T11" s="26">
+      <c r="T11" s="25">
         <v>44985.885740740741</v>
       </c>
-      <c r="U11" s="22">
+      <c r="U11" s="21">
         <v>32.938851</v>
       </c>
-      <c r="V11" s="22">
+      <c r="V11" s="21">
         <v>-117.768916</v>
       </c>
-      <c r="W11" s="28">
+      <c r="W11" s="27">
         <v>0.59861111111111109</v>
       </c>
-      <c r="X11" s="28">
+      <c r="X11" s="27">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="Y11" s="22"/>
-      <c r="Z11" s="22"/>
-      <c r="AA11" s="22"/>
+      <c r="Y11" s="21"/>
+      <c r="Z11" s="21"/>
+      <c r="AA11" s="21"/>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
@@ -1573,70 +1639,70 @@
       <c r="Z13" s="1"/>
       <c r="AA13" s="1"/>
     </row>
-    <row r="14" spans="1:27" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="22">
+    <row r="14" spans="1:27" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="21">
         <v>9</v>
       </c>
-      <c r="B14" s="22"/>
-      <c r="C14" s="22">
+      <c r="B14" s="21"/>
+      <c r="C14" s="21">
         <v>6</v>
       </c>
-      <c r="D14" s="22">
+      <c r="D14" s="21">
         <v>1</v>
       </c>
-      <c r="E14" s="23">
+      <c r="E14" s="22">
         <v>44985</v>
       </c>
-      <c r="F14" s="24"/>
-      <c r="G14" s="22">
+      <c r="F14" s="23"/>
+      <c r="G14" s="21">
         <v>32.912492</v>
       </c>
-      <c r="H14" s="22">
+      <c r="H14" s="21">
         <v>-117.69094200000001</v>
       </c>
-      <c r="I14" s="23"/>
-      <c r="J14" s="27"/>
-      <c r="K14" s="22"/>
-      <c r="L14" s="22"/>
-      <c r="M14" s="22">
+      <c r="I14" s="22"/>
+      <c r="J14" s="26"/>
+      <c r="K14" s="21"/>
+      <c r="L14" s="21"/>
+      <c r="M14" s="21">
         <v>4</v>
       </c>
-      <c r="N14" s="22" t="s">
+      <c r="N14" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="O14" s="25">
+      <c r="O14" s="24">
         <v>300434066489180</v>
       </c>
-      <c r="P14" s="25" t="s">
+      <c r="P14" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="Q14" s="26">
+      <c r="Q14" s="25">
         <v>44985.715925925928</v>
       </c>
-      <c r="R14" s="22">
+      <c r="R14" s="21">
         <v>32.911934000000002</v>
       </c>
-      <c r="S14" s="22">
+      <c r="S14" s="21">
         <v>-117.691322</v>
       </c>
-      <c r="T14" s="26">
+      <c r="T14" s="25">
         <v>44985.788761574076</v>
       </c>
-      <c r="U14" s="22">
+      <c r="U14" s="21">
         <v>32.910586000000002</v>
       </c>
-      <c r="V14" s="22">
+      <c r="V14" s="21">
         <v>-117.69389</v>
       </c>
-      <c r="W14" s="28">
+      <c r="W14" s="27">
         <v>0.59861111111111109</v>
       </c>
-      <c r="X14" s="28">
+      <c r="X14" s="27">
         <v>7.3611111111111113E-2</v>
       </c>
-      <c r="Y14" s="22"/>
-      <c r="Z14" s="22"/>
-      <c r="AA14" s="22" t="s">
+      <c r="Y14" s="21"/>
+      <c r="Z14" s="21"/>
+      <c r="AA14" s="21" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1717,127 +1783,127 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:27" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="22">
+    <row r="16" spans="1:27" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="21">
         <v>11</v>
       </c>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22">
+      <c r="B16" s="21"/>
+      <c r="C16" s="21">
         <v>4</v>
       </c>
-      <c r="D16" s="22">
+      <c r="D16" s="21">
         <v>1</v>
       </c>
-      <c r="E16" s="23">
+      <c r="E16" s="22">
         <v>45084</v>
       </c>
-      <c r="F16" s="24"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="22"/>
-      <c r="M16" s="22">
+      <c r="F16" s="23"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="21"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="26"/>
+      <c r="K16" s="21"/>
+      <c r="L16" s="21"/>
+      <c r="M16" s="21">
         <v>1</v>
       </c>
-      <c r="N16" s="22" t="s">
+      <c r="N16" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="O16" s="25">
+      <c r="O16" s="24">
         <v>300434066482170</v>
       </c>
-      <c r="P16" s="25" t="s">
+      <c r="P16" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="Q16" s="26">
+      <c r="Q16" s="25">
         <v>45084.72278935185</v>
       </c>
-      <c r="R16" s="22">
+      <c r="R16" s="21">
         <v>32.907145</v>
       </c>
-      <c r="S16" s="22">
+      <c r="S16" s="21">
         <v>-117.747221</v>
       </c>
-      <c r="T16" s="26">
+      <c r="T16" s="25">
         <v>45085.253900462965</v>
       </c>
-      <c r="U16" s="22">
+      <c r="U16" s="21">
         <v>32.939883999999999</v>
       </c>
-      <c r="V16" s="22">
+      <c r="V16" s="21">
         <v>-117.83437499999999</v>
       </c>
-      <c r="W16" s="28">
+      <c r="W16" s="27">
         <v>0.52916666666666667</v>
       </c>
-      <c r="X16" s="28">
+      <c r="X16" s="27">
         <v>0.12291666666666667</v>
       </c>
-      <c r="Y16" s="22"/>
-      <c r="Z16" s="22"/>
-      <c r="AA16" s="22"/>
-    </row>
-    <row r="17" spans="1:27" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="22">
+      <c r="Y16" s="21"/>
+      <c r="Z16" s="21"/>
+      <c r="AA16" s="21"/>
+    </row>
+    <row r="17" spans="1:27" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="21">
         <v>11</v>
       </c>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22">
+      <c r="B17" s="21"/>
+      <c r="C17" s="21">
         <v>4</v>
       </c>
-      <c r="D17" s="22">
+      <c r="D17" s="21">
         <v>2</v>
       </c>
-      <c r="E17" s="23">
+      <c r="E17" s="22">
         <v>45084</v>
       </c>
-      <c r="F17" s="24"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="27"/>
-      <c r="K17" s="22"/>
-      <c r="L17" s="22"/>
-      <c r="M17" s="22">
+      <c r="F17" s="23"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="21"/>
+      <c r="L17" s="21"/>
+      <c r="M17" s="21">
         <v>1</v>
       </c>
-      <c r="N17" s="22" t="s">
+      <c r="N17" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="O17" s="25">
+      <c r="O17" s="24">
         <v>300434066482170</v>
       </c>
-      <c r="P17" s="25" t="s">
+      <c r="P17" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="Q17" s="30">
+      <c r="Q17" s="29">
         <v>45085.26767361111</v>
       </c>
-      <c r="R17" s="31">
+      <c r="R17" s="30">
         <v>32.939607000000002</v>
       </c>
-      <c r="S17" s="31">
+      <c r="S17" s="30">
         <v>-117.834576</v>
       </c>
-      <c r="T17" s="30">
+      <c r="T17" s="29">
         <v>45085.753796296296</v>
       </c>
-      <c r="U17" s="31">
+      <c r="U17" s="30">
         <v>32.963126000000003</v>
       </c>
-      <c r="V17" s="31">
+      <c r="V17" s="30">
         <v>-117.875584</v>
       </c>
-      <c r="W17" s="28">
+      <c r="W17" s="27">
         <v>0.52916666666666667</v>
       </c>
-      <c r="X17" s="28">
+      <c r="X17" s="27">
         <v>0.12291666666666667</v>
       </c>
-      <c r="Y17" s="22"/>
-      <c r="Z17" s="22"/>
-      <c r="AA17" s="22"/>
+      <c r="Y17" s="21"/>
+      <c r="Z17" s="21"/>
+      <c r="AA17" s="21"/>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
@@ -1961,975 +2027,975 @@
       <c r="Z19" s="1"/>
       <c r="AA19" s="1"/>
     </row>
-    <row r="20" spans="1:27" s="29" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="22">
+    <row r="20" spans="1:27" s="28" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="21">
         <v>13</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="22">
+      <c r="C20" s="21">
         <v>6</v>
       </c>
-      <c r="D20" s="22">
+      <c r="D20" s="21">
         <v>1</v>
       </c>
-      <c r="E20" s="23">
+      <c r="E20" s="22">
         <v>45176</v>
       </c>
-      <c r="F20" s="24">
+      <c r="F20" s="23">
         <v>0.37708333333333338</v>
       </c>
-      <c r="G20" s="22">
+      <c r="G20" s="21">
         <v>32.910367999999998</v>
       </c>
-      <c r="H20" s="22">
+      <c r="H20" s="21">
         <v>-117.737223</v>
       </c>
-      <c r="I20" s="23">
+      <c r="I20" s="22">
         <v>45180</v>
       </c>
-      <c r="J20" s="27"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
-      <c r="M20" s="22">
+      <c r="J20" s="26"/>
+      <c r="K20" s="21"/>
+      <c r="L20" s="21"/>
+      <c r="M20" s="21">
         <v>4</v>
       </c>
-      <c r="N20" s="22" t="s">
+      <c r="N20" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="O20" s="25">
+      <c r="O20" s="24">
         <v>300434066480130</v>
       </c>
-      <c r="P20" s="25" t="s">
+      <c r="P20" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="Q20" s="30">
+      <c r="Q20" s="29">
         <v>45176.681122685186</v>
       </c>
-      <c r="R20" s="31">
+      <c r="R20" s="30">
         <v>32.911997999999997</v>
       </c>
-      <c r="S20" s="31">
+      <c r="S20" s="30">
         <v>-117.736034</v>
       </c>
-      <c r="T20" s="30">
+      <c r="T20" s="29">
         <v>45180.389189814814</v>
       </c>
-      <c r="U20" s="32">
+      <c r="U20" s="31">
         <v>32.880761</v>
       </c>
-      <c r="V20" s="32">
+      <c r="V20" s="31">
         <v>-117.434878</v>
       </c>
-      <c r="W20" s="28">
+      <c r="W20" s="27">
         <v>0.57361111111111118</v>
       </c>
-      <c r="X20" s="28">
+      <c r="X20" s="27">
         <v>6.2847222222222221E-2</v>
       </c>
-      <c r="Y20" s="22"/>
-      <c r="Z20" s="22"/>
-      <c r="AA20" s="22"/>
-    </row>
-    <row r="21" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="1">
+      <c r="Y20" s="21"/>
+      <c r="Z20" s="21"/>
+      <c r="AA20" s="21"/>
+    </row>
+    <row r="21" spans="1:27" s="40" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="33">
         <v>14</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21" s="33">
         <v>4</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="33">
         <v>1</v>
       </c>
-      <c r="E21" s="2">
+      <c r="E21" s="34">
         <v>45203</v>
       </c>
-      <c r="F21" s="3">
+      <c r="F21" s="35">
         <v>0.29722222222222222</v>
       </c>
-      <c r="G21" s="1">
+      <c r="G21" s="33">
         <v>38.709972999999998</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H21" s="33">
         <v>-64.031019999999998</v>
       </c>
-      <c r="I21" s="2">
+      <c r="I21" s="34">
         <v>45204</v>
       </c>
-      <c r="J21" s="6">
+      <c r="J21" s="38">
         <v>0.61805555555555558</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="33">
         <v>38.864894999999997</v>
       </c>
-      <c r="L21" s="1">
+      <c r="L21" s="33">
         <v>-64.055637000000004</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M21" s="33">
         <v>1</v>
       </c>
-      <c r="N21" s="1" t="s">
+      <c r="N21" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="O21" s="4">
+      <c r="O21" s="36">
         <v>300434066489180</v>
       </c>
-      <c r="P21" s="4" t="s">
+      <c r="P21" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="Q21" s="5">
+      <c r="Q21" s="37">
         <v>45203.334583333337</v>
       </c>
-      <c r="R21" s="11">
+      <c r="R21" s="41">
         <v>38.726599999999998</v>
       </c>
-      <c r="S21" s="11">
+      <c r="S21" s="41">
         <v>-64.021100000000004</v>
       </c>
-      <c r="T21" s="5">
+      <c r="T21" s="37">
         <v>45204.785219907404</v>
       </c>
-      <c r="U21" s="8">
+      <c r="U21" s="40">
         <v>38.864600000000003</v>
       </c>
-      <c r="V21" s="8">
+      <c r="V21" s="40">
         <v>-64.055627999999999</v>
       </c>
-      <c r="W21" s="7">
+      <c r="W21" s="39">
         <v>0.42708333333333331</v>
       </c>
-      <c r="X21" s="7">
+      <c r="X21" s="39">
         <v>0.91180555555555554</v>
       </c>
-      <c r="Y21" s="1">
+      <c r="Y21" s="33">
         <v>300</v>
       </c>
-      <c r="Z21" s="1">
+      <c r="Z21" s="33">
         <v>4</v>
       </c>
-      <c r="AA21" s="1" t="s">
+      <c r="AA21" s="33" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="22" spans="1:27" s="29" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="22">
+    <row r="22" spans="1:27" s="50" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="42">
         <v>15</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22" s="42">
         <v>5</v>
       </c>
-      <c r="D22" s="22">
+      <c r="D22" s="42">
         <v>1</v>
       </c>
-      <c r="E22" s="23">
+      <c r="E22" s="43">
         <v>45203</v>
       </c>
-      <c r="F22" s="24">
+      <c r="F22" s="44">
         <v>0.29444444444444445</v>
       </c>
-      <c r="G22" s="22">
+      <c r="G22" s="42">
         <v>38.708799999999997</v>
       </c>
-      <c r="H22" s="22">
+      <c r="H22" s="42">
         <v>-64.031542999999999</v>
       </c>
-      <c r="I22" s="23">
+      <c r="I22" s="43">
         <v>45205</v>
       </c>
-      <c r="J22" s="27">
+      <c r="J22" s="45">
         <v>0.37847222222222227</v>
       </c>
-      <c r="K22" s="22">
+      <c r="K22" s="42">
         <v>38.943779999999997</v>
       </c>
-      <c r="L22" s="22">
+      <c r="L22" s="42">
         <v>-64.196479999999994</v>
       </c>
-      <c r="M22" s="22">
+      <c r="M22" s="42">
         <v>3</v>
       </c>
-      <c r="N22" s="22" t="s">
+      <c r="N22" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="O22" s="25">
+      <c r="O22" s="46">
         <v>300434066482170</v>
       </c>
-      <c r="P22" s="25" t="s">
+      <c r="P22" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="Q22" s="26">
+      <c r="Q22" s="47">
         <v>45203.535277777781</v>
       </c>
-      <c r="R22" s="32">
+      <c r="R22" s="48">
         <v>38.722087999999999</v>
       </c>
-      <c r="S22" s="32">
+      <c r="S22" s="48">
         <v>-64.021294999999995</v>
       </c>
-      <c r="T22" s="26">
+      <c r="T22" s="47">
         <v>45204.719074074077</v>
       </c>
-      <c r="U22" s="32">
+      <c r="U22" s="48">
         <v>38.866824999999999</v>
       </c>
-      <c r="V22" s="32">
+      <c r="V22" s="48">
         <v>-64.043930000000003</v>
       </c>
-      <c r="W22" s="28">
+      <c r="W22" s="49">
         <v>0.42708333333333331</v>
       </c>
-      <c r="X22" s="28">
+      <c r="X22" s="49">
         <v>0.91180555555555554</v>
       </c>
-      <c r="Y22" s="22">
+      <c r="Y22" s="42">
         <v>300</v>
       </c>
-      <c r="Z22" s="22">
+      <c r="Z22" s="42">
         <v>4</v>
       </c>
-      <c r="AA22" s="22" t="s">
+      <c r="AA22" s="42" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:27" s="29" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="22">
+    <row r="23" spans="1:27" s="50" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="42">
         <v>15</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="22">
+      <c r="C23" s="42">
         <v>5</v>
       </c>
-      <c r="D23" s="22">
+      <c r="D23" s="42">
         <v>2</v>
       </c>
-      <c r="E23" s="23">
+      <c r="E23" s="43">
         <v>45203</v>
       </c>
-      <c r="F23" s="24">
+      <c r="F23" s="44">
         <v>0.29444444444444445</v>
       </c>
-      <c r="G23" s="22">
+      <c r="G23" s="42">
         <v>38.708799999999997</v>
       </c>
-      <c r="H23" s="22">
+      <c r="H23" s="42">
         <v>-64.031542999999999</v>
       </c>
-      <c r="I23" s="23">
+      <c r="I23" s="43">
         <v>45205</v>
       </c>
-      <c r="J23" s="27">
+      <c r="J23" s="45">
         <v>0.37847222222222227</v>
       </c>
-      <c r="K23" s="22">
+      <c r="K23" s="42">
         <v>38.943779999999997</v>
       </c>
-      <c r="L23" s="22">
+      <c r="L23" s="42">
         <v>-64.196479999999994</v>
       </c>
-      <c r="M23" s="22">
+      <c r="M23" s="42">
         <v>3</v>
       </c>
-      <c r="N23" s="22" t="s">
+      <c r="N23" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="O23" s="25">
+      <c r="O23" s="46">
         <v>300434066482170</v>
       </c>
-      <c r="P23" s="25" t="s">
+      <c r="P23" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="Q23" s="30">
+      <c r="Q23" s="51">
         <v>45204.812939814816</v>
       </c>
-      <c r="R23" s="32">
+      <c r="R23" s="48">
         <v>38.887227000000003</v>
       </c>
-      <c r="S23" s="32">
+      <c r="S23" s="48">
         <v>-64.073801000000003</v>
       </c>
-      <c r="T23" s="30">
+      <c r="T23" s="51">
         <v>45205.389224537037</v>
       </c>
-      <c r="U23" s="32">
+      <c r="U23" s="48">
         <v>38.930204000000003</v>
       </c>
-      <c r="V23" s="32">
+      <c r="V23" s="48">
         <v>-64.167721999999998</v>
       </c>
-      <c r="W23" s="28">
+      <c r="W23" s="49">
         <v>0.42708333333333331</v>
       </c>
-      <c r="X23" s="28">
+      <c r="X23" s="49">
         <v>0.91180555555555554</v>
       </c>
-      <c r="Y23" s="22">
+      <c r="Y23" s="42">
         <v>300</v>
       </c>
-      <c r="Z23" s="22">
+      <c r="Z23" s="42">
         <v>4</v>
       </c>
-      <c r="AA23" s="22" t="s">
+      <c r="AA23" s="42" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="24" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="1">
+    <row r="24" spans="1:27" s="40" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="33">
         <v>16</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="C24" s="1">
+      <c r="C24" s="33">
         <v>6</v>
       </c>
-      <c r="D24" s="1">
+      <c r="D24" s="33">
         <v>1</v>
       </c>
-      <c r="E24" s="2">
+      <c r="E24" s="34">
         <v>45203</v>
       </c>
-      <c r="F24" s="3">
+      <c r="F24" s="35">
         <v>0.3034722222222222</v>
       </c>
-      <c r="G24" s="1">
+      <c r="G24" s="33">
         <v>38.710590000000003</v>
       </c>
-      <c r="H24" s="1">
+      <c r="H24" s="33">
         <v>-64.028107000000006</v>
       </c>
-      <c r="I24" s="2">
+      <c r="I24" s="34">
         <v>45205</v>
       </c>
-      <c r="J24" s="6">
+      <c r="J24" s="38">
         <v>0.35416666666666669</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="33">
         <v>38.930132999999998</v>
       </c>
-      <c r="L24" s="1">
+      <c r="L24" s="33">
         <v>-64.154741999999999</v>
       </c>
-      <c r="M24" s="1">
+      <c r="M24" s="33">
         <v>4</v>
       </c>
-      <c r="N24" s="1" t="s">
+      <c r="N24" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="O24" s="4">
+      <c r="O24" s="36">
         <v>300434066480130</v>
       </c>
-      <c r="P24" s="4" t="s">
+      <c r="P24" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="Q24" s="9">
+      <c r="Q24" s="52">
         <v>45203.528344907405</v>
       </c>
-      <c r="R24" s="11">
+      <c r="R24" s="41">
         <v>38.720514999999999</v>
       </c>
-      <c r="S24" s="11">
+      <c r="S24" s="41">
         <v>-64.019482999999994</v>
       </c>
-      <c r="T24" s="9">
+      <c r="T24" s="52">
         <v>45204.712129629632</v>
       </c>
-      <c r="U24" s="11">
+      <c r="U24" s="41">
         <v>38.873122000000002</v>
       </c>
-      <c r="V24" s="11">
+      <c r="V24" s="41">
         <v>-64.033095000000003</v>
       </c>
-      <c r="W24" s="7">
+      <c r="W24" s="39">
         <v>0.42708333333333331</v>
       </c>
-      <c r="X24" s="7">
+      <c r="X24" s="39">
         <v>0.91180555555555554</v>
       </c>
-      <c r="Y24" s="1">
+      <c r="Y24" s="33">
         <v>300</v>
       </c>
-      <c r="Z24" s="1">
+      <c r="Z24" s="33">
         <v>4</v>
       </c>
-      <c r="AA24" s="1"/>
-    </row>
-    <row r="25" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="1">
+      <c r="AA24" s="33"/>
+    </row>
+    <row r="25" spans="1:27" s="40" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="33">
         <v>16</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" s="33">
         <v>6</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D25" s="33">
         <v>2</v>
       </c>
-      <c r="E25" s="2">
+      <c r="E25" s="34">
         <v>45203</v>
       </c>
-      <c r="F25" s="3">
+      <c r="F25" s="35">
         <v>0.3034722222222222</v>
       </c>
-      <c r="G25" s="1">
+      <c r="G25" s="33">
         <v>38.710590000000003</v>
       </c>
-      <c r="H25" s="1">
+      <c r="H25" s="33">
         <v>-64.028107000000006</v>
       </c>
-      <c r="I25" s="2">
+      <c r="I25" s="34">
         <v>45205</v>
       </c>
-      <c r="J25" s="6">
+      <c r="J25" s="38">
         <v>0.35416666666666669</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="33">
         <v>38.930132999999998</v>
       </c>
-      <c r="L25" s="1">
+      <c r="L25" s="33">
         <v>-64.154741999999999</v>
       </c>
-      <c r="M25" s="1">
+      <c r="M25" s="33">
         <v>4</v>
       </c>
-      <c r="N25" s="1" t="s">
+      <c r="N25" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="O25" s="4">
+      <c r="O25" s="36">
         <v>300434066480130</v>
       </c>
-      <c r="P25" s="4" t="s">
+      <c r="P25" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="Q25" s="9">
+      <c r="Q25" s="52">
         <v>45204.771168981482</v>
       </c>
-      <c r="R25" s="11">
+      <c r="R25" s="41">
         <v>38.886073000000003</v>
       </c>
-      <c r="S25" s="11">
+      <c r="S25" s="41">
         <v>-64.054066000000006</v>
       </c>
-      <c r="T25" s="9">
+      <c r="T25" s="52">
         <v>45205.392685185187</v>
       </c>
-      <c r="U25" s="11">
+      <c r="U25" s="41">
         <v>38.916741999999999</v>
       </c>
-      <c r="V25" s="11">
+      <c r="V25" s="41">
         <v>-64.137314000000003</v>
       </c>
-      <c r="W25" s="7">
+      <c r="W25" s="39">
         <v>0.42708333333333331</v>
       </c>
-      <c r="X25" s="7">
+      <c r="X25" s="39">
         <v>0.91180555555555554</v>
       </c>
-      <c r="Y25" s="1">
+      <c r="Y25" s="33">
         <v>300</v>
       </c>
-      <c r="Z25" s="1">
+      <c r="Z25" s="33">
         <v>4</v>
       </c>
-      <c r="AA25" s="1"/>
-    </row>
-    <row r="26" spans="1:27" s="29" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="22">
+      <c r="AA25" s="33"/>
+    </row>
+    <row r="26" spans="1:27" s="50" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="42">
         <v>17</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="C26" s="22">
+      <c r="C26" s="42">
         <v>6</v>
       </c>
-      <c r="D26" s="22">
+      <c r="D26" s="42">
         <v>1</v>
       </c>
-      <c r="E26" s="23">
+      <c r="E26" s="43">
         <v>45207</v>
       </c>
-      <c r="F26" s="24">
+      <c r="F26" s="44">
         <v>0.92152777777777783</v>
       </c>
-      <c r="G26" s="22">
+      <c r="G26" s="42">
         <v>38.767780000000002</v>
       </c>
-      <c r="H26" s="22">
+      <c r="H26" s="42">
         <v>-63.738374</v>
       </c>
-      <c r="I26" s="23">
+      <c r="I26" s="43">
         <v>45210</v>
       </c>
-      <c r="J26" s="27">
+      <c r="J26" s="45">
         <v>0.40625</v>
       </c>
-      <c r="K26" s="29">
+      <c r="K26" s="50">
         <v>38.954067000000002</v>
       </c>
-      <c r="L26" s="22">
+      <c r="L26" s="42">
         <v>-63.862921999999998</v>
       </c>
-      <c r="M26" s="22">
+      <c r="M26" s="42">
         <v>4</v>
       </c>
-      <c r="N26" s="22" t="s">
+      <c r="N26" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="O26" s="25">
+      <c r="O26" s="46">
         <v>300434066480130</v>
       </c>
-      <c r="P26" s="25" t="s">
+      <c r="P26" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="Q26" s="30">
+      <c r="Q26" s="51">
         <v>45208.132511574076</v>
       </c>
-      <c r="R26" s="33">
+      <c r="R26" s="53">
         <v>38.769841999999997</v>
       </c>
-      <c r="S26" s="33">
+      <c r="S26" s="53">
         <v>-63.7483</v>
       </c>
-      <c r="T26" s="30">
+      <c r="T26" s="51">
         <v>45208.63921296296</v>
       </c>
-      <c r="U26" s="33">
+      <c r="U26" s="53">
         <v>38.832385000000002</v>
       </c>
-      <c r="V26" s="33">
+      <c r="V26" s="53">
         <v>-63.796340000000001</v>
       </c>
-      <c r="W26" s="28">
+      <c r="W26" s="49">
         <v>0.42708333333333298</v>
       </c>
-      <c r="X26" s="28">
+      <c r="X26" s="49">
         <v>0.91180555555555598</v>
       </c>
-      <c r="Y26" s="22">
+      <c r="Y26" s="42">
         <v>200</v>
       </c>
-      <c r="Z26" s="22">
+      <c r="Z26" s="42">
         <v>4</v>
       </c>
-      <c r="AA26" s="22"/>
-    </row>
-    <row r="27" spans="1:27" s="29" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="22">
+      <c r="AA26" s="42"/>
+    </row>
+    <row r="27" spans="1:27" s="50" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="42">
         <v>17</v>
       </c>
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="C27" s="22">
+      <c r="C27" s="42">
         <v>6</v>
       </c>
-      <c r="D27" s="22">
+      <c r="D27" s="42">
         <v>2</v>
       </c>
-      <c r="E27" s="23">
+      <c r="E27" s="43">
         <v>45207</v>
       </c>
-      <c r="F27" s="24">
+      <c r="F27" s="44">
         <v>0.92152777777777783</v>
       </c>
-      <c r="G27" s="22">
+      <c r="G27" s="42">
         <v>38.767780000000002</v>
       </c>
-      <c r="H27" s="22">
+      <c r="H27" s="42">
         <v>-63.738374</v>
       </c>
-      <c r="I27" s="23">
+      <c r="I27" s="43">
         <v>45210</v>
       </c>
-      <c r="J27" s="27">
+      <c r="J27" s="45">
         <v>0.40625</v>
       </c>
-      <c r="K27" s="29">
+      <c r="K27" s="50">
         <v>38.954067000000002</v>
       </c>
-      <c r="L27" s="22">
+      <c r="L27" s="42">
         <v>-63.862921999999998</v>
       </c>
-      <c r="M27" s="22">
+      <c r="M27" s="42">
         <v>4</v>
       </c>
-      <c r="N27" s="22" t="s">
+      <c r="N27" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="O27" s="25">
+      <c r="O27" s="46">
         <v>300434066480130</v>
       </c>
-      <c r="P27" s="25" t="s">
+      <c r="P27" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="Q27" s="30">
+      <c r="Q27" s="51">
         <v>45208.771828703706</v>
       </c>
-      <c r="R27" s="33">
+      <c r="R27" s="53">
         <v>38.857106999999999</v>
       </c>
-      <c r="S27" s="33">
+      <c r="S27" s="53">
         <v>-63.781923999999997</v>
       </c>
-      <c r="T27" s="30">
+      <c r="T27" s="51">
         <v>45209.656574074077</v>
       </c>
-      <c r="U27" s="33">
+      <c r="U27" s="53">
         <v>38.923247000000003</v>
       </c>
-      <c r="V27" s="33">
+      <c r="V27" s="53">
         <v>-63.812421999999998</v>
       </c>
-      <c r="W27" s="28">
+      <c r="W27" s="49">
         <v>0.42708333333333298</v>
       </c>
-      <c r="X27" s="28">
+      <c r="X27" s="49">
         <v>0.91180555555555598</v>
       </c>
-      <c r="Y27" s="22">
+      <c r="Y27" s="42">
         <v>300</v>
       </c>
-      <c r="Z27" s="22">
+      <c r="Z27" s="42">
         <v>4</v>
       </c>
-      <c r="AA27" s="22"/>
-    </row>
-    <row r="28" spans="1:27" s="29" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="22">
+      <c r="AA27" s="42"/>
+    </row>
+    <row r="28" spans="1:27" s="50" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="42">
         <v>17</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="C28" s="22">
+      <c r="C28" s="42">
         <v>6</v>
       </c>
-      <c r="D28" s="22">
+      <c r="D28" s="42">
         <v>3</v>
       </c>
-      <c r="E28" s="23">
+      <c r="E28" s="43">
         <v>45207</v>
       </c>
-      <c r="F28" s="24">
+      <c r="F28" s="44">
         <v>0.92152777777777783</v>
       </c>
-      <c r="G28" s="22">
+      <c r="G28" s="42">
         <v>38.767780000000002</v>
       </c>
-      <c r="H28" s="22">
+      <c r="H28" s="42">
         <v>-63.738374</v>
       </c>
-      <c r="I28" s="23">
+      <c r="I28" s="43">
         <v>45210</v>
       </c>
-      <c r="J28" s="27">
+      <c r="J28" s="45">
         <v>0.40625</v>
       </c>
-      <c r="K28" s="29">
+      <c r="K28" s="50">
         <v>38.954067000000002</v>
       </c>
-      <c r="L28" s="22">
+      <c r="L28" s="42">
         <v>-63.862921999999998</v>
       </c>
-      <c r="M28" s="22">
+      <c r="M28" s="42">
         <v>4</v>
       </c>
-      <c r="N28" s="22" t="s">
+      <c r="N28" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="O28" s="25">
+      <c r="O28" s="46">
         <v>300434066480130</v>
       </c>
-      <c r="P28" s="25" t="s">
+      <c r="P28" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="Q28" s="30">
+      <c r="Q28" s="51">
         <v>45209.750567129631</v>
       </c>
-      <c r="R28" s="33">
+      <c r="R28" s="53">
         <v>38.923658000000003</v>
       </c>
-      <c r="S28" s="33">
+      <c r="S28" s="53">
         <v>-63.819659000000001</v>
       </c>
-      <c r="T28" s="30">
+      <c r="T28" s="51">
         <v>45210.542002314818</v>
       </c>
-      <c r="U28" s="33">
+      <c r="U28" s="53">
         <v>38.940576999999998</v>
       </c>
-      <c r="V28" s="33">
+      <c r="V28" s="53">
         <v>-63.867663</v>
       </c>
-      <c r="W28" s="28">
+      <c r="W28" s="49">
         <v>0.42708333333333298</v>
       </c>
-      <c r="X28" s="28">
+      <c r="X28" s="49">
         <v>0.91180555555555598</v>
       </c>
-      <c r="Y28" s="22">
+      <c r="Y28" s="42">
         <v>200</v>
       </c>
-      <c r="Z28" s="22">
+      <c r="Z28" s="42">
         <v>4</v>
       </c>
-      <c r="AA28" s="22"/>
-    </row>
-    <row r="29" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="1">
+      <c r="AA28" s="42"/>
+    </row>
+    <row r="29" spans="1:27" s="40" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="33">
         <v>18</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="C29" s="1">
+      <c r="C29" s="33">
         <v>4</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="33">
         <v>1</v>
       </c>
-      <c r="E29" s="2">
+      <c r="E29" s="34">
         <v>45207</v>
       </c>
-      <c r="F29" s="3">
+      <c r="F29" s="35">
         <v>0.9243055555555556</v>
       </c>
-      <c r="G29" s="1">
+      <c r="G29" s="33">
         <v>38.768692000000001</v>
       </c>
-      <c r="H29" s="1">
+      <c r="H29" s="33">
         <v>-63.73818</v>
       </c>
-      <c r="I29" s="2">
+      <c r="I29" s="34">
         <v>45210</v>
       </c>
-      <c r="J29" s="6">
+      <c r="J29" s="38">
         <v>0.31180555555555556</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="33">
         <v>38.979595000000003</v>
       </c>
-      <c r="L29" s="1">
+      <c r="L29" s="33">
         <v>-63.837929000000003</v>
       </c>
-      <c r="M29" s="1">
+      <c r="M29" s="33">
         <v>1</v>
       </c>
-      <c r="N29" s="1" t="s">
+      <c r="N29" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="O29" s="4">
+      <c r="O29" s="36">
         <v>300434066489180</v>
       </c>
-      <c r="P29" s="4" t="s">
+      <c r="P29" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="Q29" s="9">
+      <c r="Q29" s="52">
         <v>45208.1325</v>
       </c>
-      <c r="R29" s="12">
+      <c r="R29" s="54">
         <v>38.770648000000001</v>
       </c>
-      <c r="S29" s="12">
+      <c r="S29" s="54">
         <v>-63.747129000000001</v>
       </c>
-      <c r="T29" s="9">
+      <c r="T29" s="52">
         <v>45208.687939814816</v>
       </c>
-      <c r="U29" s="12">
+      <c r="U29" s="54">
         <v>38.808157999999999</v>
       </c>
-      <c r="V29" s="12">
+      <c r="V29" s="54">
         <v>-63.765051999999997</v>
       </c>
-      <c r="W29" s="7">
+      <c r="W29" s="39">
         <v>0.42708333333333298</v>
       </c>
-      <c r="X29" s="7">
+      <c r="X29" s="39">
         <v>0.91180555555555598</v>
       </c>
-      <c r="Y29" s="1">
+      <c r="Y29" s="33">
         <v>300</v>
       </c>
-      <c r="Z29" s="1">
+      <c r="Z29" s="33">
         <v>4</v>
       </c>
-      <c r="AA29" s="1" t="s">
+      <c r="AA29" s="33" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="1">
+    <row r="30" spans="1:27" s="40" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="33">
         <v>18</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="C30" s="1">
+      <c r="C30" s="33">
         <v>4</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="33">
         <v>2</v>
       </c>
-      <c r="E30" s="2">
+      <c r="E30" s="34">
         <v>45207</v>
       </c>
-      <c r="F30" s="3">
+      <c r="F30" s="35">
         <v>0.9243055555555556</v>
       </c>
-      <c r="G30" s="1">
+      <c r="G30" s="33">
         <v>38.768692000000001</v>
       </c>
-      <c r="H30" s="1">
+      <c r="H30" s="33">
         <v>-63.73818</v>
       </c>
-      <c r="I30" s="2">
+      <c r="I30" s="34">
         <v>45210</v>
       </c>
-      <c r="J30" s="6">
+      <c r="J30" s="38">
         <v>0.31180555555555556</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="33">
         <v>38.979595000000003</v>
       </c>
-      <c r="L30" s="1">
+      <c r="L30" s="33">
         <v>-63.837929000000003</v>
       </c>
-      <c r="M30" s="1">
+      <c r="M30" s="33">
         <v>2</v>
       </c>
-      <c r="N30" s="1" t="s">
+      <c r="N30" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="O30" s="4">
+      <c r="O30" s="36">
         <v>300434066489180</v>
       </c>
-      <c r="P30" s="4" t="s">
+      <c r="P30" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="Q30" s="9">
+      <c r="Q30" s="52">
         <v>45208.764548611114</v>
       </c>
-      <c r="R30" s="12">
+      <c r="R30" s="54">
         <v>38.822692000000004</v>
       </c>
-      <c r="S30" s="12">
+      <c r="S30" s="54">
         <v>-63.766671000000002</v>
       </c>
-      <c r="T30" s="9">
+      <c r="T30" s="52">
         <v>45209.63921296296</v>
       </c>
-      <c r="U30" s="12">
+      <c r="U30" s="54">
         <v>38.928795999999998</v>
       </c>
-      <c r="V30" s="12">
+      <c r="V30" s="54">
         <v>-63.821711999999998</v>
       </c>
-      <c r="W30" s="7">
+      <c r="W30" s="39">
         <v>0.42708333333333298</v>
       </c>
-      <c r="X30" s="7">
+      <c r="X30" s="39">
         <v>0.91180555555555598</v>
       </c>
-      <c r="Y30" s="1">
+      <c r="Y30" s="33">
         <v>200</v>
       </c>
-      <c r="Z30" s="1">
+      <c r="Z30" s="33">
         <v>4</v>
       </c>
-      <c r="AA30" s="1"/>
-    </row>
-    <row r="31" spans="1:27" s="29" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="22">
+      <c r="AA30" s="33"/>
+    </row>
+    <row r="31" spans="1:27" s="50" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="42">
         <v>19</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="42" t="s">
         <v>44</v>
       </c>
-      <c r="C31" s="22">
+      <c r="C31" s="42">
         <v>5</v>
       </c>
-      <c r="D31" s="22">
+      <c r="D31" s="42">
         <v>1</v>
       </c>
-      <c r="E31" s="23">
+      <c r="E31" s="43">
         <v>45208</v>
       </c>
-      <c r="F31" s="24">
+      <c r="F31" s="44">
         <v>0.59722222222222221</v>
       </c>
-      <c r="G31" s="22">
+      <c r="G31" s="42">
         <v>38.826842999999997</v>
       </c>
-      <c r="H31" s="22">
+      <c r="H31" s="42">
         <v>-63.845635000000001</v>
       </c>
-      <c r="I31" s="23">
+      <c r="I31" s="43">
         <v>45209</v>
       </c>
-      <c r="J31" s="27">
+      <c r="J31" s="45">
         <v>0.36805555555555558</v>
       </c>
-      <c r="K31" s="22">
+      <c r="K31" s="42">
         <v>38.862192</v>
       </c>
-      <c r="L31" s="22">
+      <c r="L31" s="42">
         <v>-63.908256999999999</v>
       </c>
-      <c r="M31" s="22">
+      <c r="M31" s="42">
         <v>3</v>
       </c>
-      <c r="N31" s="22" t="s">
+      <c r="N31" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="O31" s="25">
+      <c r="O31" s="46">
         <v>300434066482170</v>
       </c>
-      <c r="P31" s="25" t="s">
+      <c r="P31" s="46" t="s">
         <v>38</v>
       </c>
-      <c r="Q31" s="30">
+      <c r="Q31" s="51">
         <v>45208.77138888889</v>
       </c>
-      <c r="R31" s="33">
+      <c r="R31" s="53">
         <v>38.827702000000002</v>
       </c>
-      <c r="S31" s="33">
+      <c r="S31" s="53">
         <v>-63.844456999999998</v>
       </c>
-      <c r="T31" s="26">
+      <c r="T31" s="47">
         <v>45209.26421296296</v>
       </c>
-      <c r="U31" s="33">
+      <c r="U31" s="53">
         <v>38.862524999999998</v>
       </c>
-      <c r="V31" s="33">
+      <c r="V31" s="53">
         <v>-63.894246000000003</v>
       </c>
-      <c r="W31" s="28">
+      <c r="W31" s="49">
         <v>0.42708333333333298</v>
       </c>
-      <c r="X31" s="28">
+      <c r="X31" s="49">
         <v>0.91180555555555598</v>
       </c>
-      <c r="Y31" s="22">
+      <c r="Y31" s="42">
         <v>100</v>
       </c>
-      <c r="Z31" s="22">
+      <c r="Z31" s="42">
         <v>4</v>
       </c>
-      <c r="AA31" s="22" t="s">
+      <c r="AA31" s="42" t="s">
         <v>51</v>
       </c>
     </row>
@@ -2959,11 +3025,17 @@
         <v>-63.903267</v>
       </c>
       <c r="I32" s="2">
-        <v>45211</v>
-      </c>
-      <c r="J32" s="6"/>
-      <c r="K32" s="1"/>
-      <c r="L32" s="1"/>
+        <v>45212</v>
+      </c>
+      <c r="J32" s="6">
+        <v>0.7680555555555556</v>
+      </c>
+      <c r="K32" s="1">
+        <v>38.899351000000003</v>
+      </c>
+      <c r="L32" s="1">
+        <v>-63.939715</v>
+      </c>
       <c r="M32" s="1">
         <v>3</v>
       </c>
@@ -2979,29 +3051,29 @@
       <c r="Q32" s="9">
         <v>45210.684594907405</v>
       </c>
-      <c r="R32" s="12">
+      <c r="R32" s="11">
         <v>38.864280999999998</v>
       </c>
-      <c r="S32" s="12">
+      <c r="S32" s="11">
         <v>-63.895504000000003</v>
       </c>
-      <c r="T32" s="9">
+      <c r="T32" s="55">
         <v>45211.541979166665</v>
       </c>
-      <c r="U32" s="42">
+      <c r="U32" s="11">
         <v>38.912925999999999</v>
       </c>
-      <c r="V32" s="42">
+      <c r="V32" s="11">
         <v>-63.895589000000001</v>
       </c>
-      <c r="W32" s="28">
+      <c r="W32" s="58">
         <v>0.42708333333333298</v>
       </c>
-      <c r="X32" s="28">
+      <c r="X32" s="58">
         <v>0.91180555555555598</v>
       </c>
       <c r="Y32" s="1">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="Z32" s="1">
         <v>4</v>
@@ -3036,11 +3108,17 @@
         <v>-63.903267</v>
       </c>
       <c r="I33" s="2">
-        <v>45211</v>
-      </c>
-      <c r="J33" s="6"/>
-      <c r="K33" s="1"/>
-      <c r="L33" s="1"/>
+        <v>45212</v>
+      </c>
+      <c r="J33" s="6">
+        <v>0.7680555555555556</v>
+      </c>
+      <c r="K33" s="1">
+        <v>38.899351000000003</v>
+      </c>
+      <c r="L33" s="1">
+        <v>-63.939715</v>
+      </c>
       <c r="M33" s="1">
         <v>3</v>
       </c>
@@ -3056,17 +3134,27 @@
       <c r="Q33" s="9">
         <v>45211.612372685187</v>
       </c>
-      <c r="R33" s="42">
+      <c r="R33" s="11">
         <v>38.929589</v>
       </c>
-      <c r="S33" s="42">
+      <c r="S33" s="11">
         <v>-63.899909000000001</v>
       </c>
-      <c r="T33" s="5"/>
-      <c r="U33" s="1"/>
-      <c r="V33" s="1"/>
-      <c r="W33" s="7"/>
-      <c r="X33" s="7"/>
+      <c r="T33" s="56">
+        <v>45212.556122685186</v>
+      </c>
+      <c r="U33" s="11">
+        <v>38.935225000000003</v>
+      </c>
+      <c r="V33" s="11">
+        <v>-63.928724000000003</v>
+      </c>
+      <c r="W33" s="39">
+        <v>0.42708333333333298</v>
+      </c>
+      <c r="X33" s="39">
+        <v>0.91180555555555598</v>
+      </c>
       <c r="Y33" s="1">
         <v>400</v>
       </c>
@@ -3075,66 +3163,88 @@
       </c>
       <c r="AA33" s="1"/>
     </row>
-    <row r="34" spans="1:27" s="29" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="22">
+    <row r="34" spans="1:27" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="21">
         <v>21</v>
       </c>
-      <c r="B34" s="22" t="s">
+      <c r="B34" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="C34" s="22">
+      <c r="C34" s="21">
         <v>4</v>
       </c>
-      <c r="D34" s="22">
+      <c r="D34" s="21">
         <v>1</v>
       </c>
-      <c r="E34" s="23">
+      <c r="E34" s="22">
         <v>45211</v>
       </c>
-      <c r="F34" s="24">
+      <c r="F34" s="23">
         <v>0.10416666666666667</v>
       </c>
-      <c r="G34" s="22">
+      <c r="G34" s="21">
         <v>38.834505</v>
       </c>
-      <c r="H34" s="22">
+      <c r="H34" s="21">
         <v>-63.75074</v>
       </c>
-      <c r="I34" s="23">
-        <v>45211</v>
-      </c>
-      <c r="J34" s="27"/>
-      <c r="K34" s="22"/>
-      <c r="L34" s="22"/>
-      <c r="M34" s="22">
+      <c r="I34" s="22">
+        <v>45212</v>
+      </c>
+      <c r="J34" s="26">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="K34" s="21">
+        <v>38.856884999999998</v>
+      </c>
+      <c r="L34" s="21">
+        <v>-63.746738999999998</v>
+      </c>
+      <c r="M34" s="21">
         <v>1</v>
       </c>
-      <c r="N34" s="22" t="s">
+      <c r="N34" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="O34" s="25">
+      <c r="O34" s="24">
         <v>300434066489180</v>
       </c>
-      <c r="P34" s="25" t="s">
+      <c r="P34" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="Q34" s="30">
+      <c r="Q34" s="29">
         <v>45211.834328703706</v>
       </c>
-      <c r="R34" s="43">
+      <c r="R34" s="32">
         <v>38.831561999999998</v>
       </c>
-      <c r="S34" s="43">
+      <c r="S34" s="32">
         <v>-63.740231999999999</v>
       </c>
-      <c r="T34" s="26"/>
-      <c r="U34" s="22"/>
-      <c r="V34" s="22"/>
-      <c r="W34" s="28"/>
-      <c r="X34" s="28"/>
-      <c r="Y34" s="22"/>
-      <c r="Z34" s="22"/>
-      <c r="AA34" s="22"/>
+      <c r="T34" s="57">
+        <v>45212.541990740741</v>
+      </c>
+      <c r="U34" s="32">
+        <v>38.884850999999998</v>
+      </c>
+      <c r="V34" s="32">
+        <v>-63.740850999999999</v>
+      </c>
+      <c r="W34" s="49">
+        <v>0.42708333333333298</v>
+      </c>
+      <c r="X34" s="49">
+        <v>0.91180555555555598</v>
+      </c>
+      <c r="Y34" s="21">
+        <v>125</v>
+      </c>
+      <c r="Z34" s="21">
+        <v>4</v>
+      </c>
+      <c r="AA34" s="21" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="35" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
@@ -3162,11 +3272,17 @@
         <v>-63.747987000000002</v>
       </c>
       <c r="I35" s="2">
-        <v>45211</v>
-      </c>
-      <c r="J35" s="6"/>
-      <c r="K35" s="1"/>
-      <c r="L35" s="1"/>
+        <v>45212</v>
+      </c>
+      <c r="J35" s="6">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="K35" s="1">
+        <v>38.856026999999997</v>
+      </c>
+      <c r="L35" s="1">
+        <v>-63.746715999999999</v>
+      </c>
       <c r="M35" s="1">
         <v>4</v>
       </c>
@@ -3182,20 +3298,36 @@
       <c r="Q35" s="9">
         <v>45211.82</v>
       </c>
-      <c r="R35" s="42">
+      <c r="R35" s="11">
         <v>38.830253999999996</v>
       </c>
-      <c r="S35" s="42">
+      <c r="S35" s="11">
         <v>-63.738950000000003</v>
       </c>
-      <c r="T35" s="5"/>
-      <c r="U35" s="1"/>
-      <c r="V35" s="1"/>
-      <c r="W35" s="7"/>
-      <c r="X35" s="7"/>
-      <c r="Y35" s="1"/>
-      <c r="Z35" s="1"/>
-      <c r="AA35" s="1"/>
+      <c r="T35" s="56">
+        <v>45212.535046296296</v>
+      </c>
+      <c r="U35" s="11">
+        <v>38.887054999999997</v>
+      </c>
+      <c r="V35" s="11">
+        <v>-63.744534000000002</v>
+      </c>
+      <c r="W35" s="59">
+        <v>0.42708333333333298</v>
+      </c>
+      <c r="X35" s="59">
+        <v>0.91180555555555598</v>
+      </c>
+      <c r="Y35" s="1">
+        <v>125</v>
+      </c>
+      <c r="Z35" s="1">
+        <v>4</v>
+      </c>
+      <c r="AA35" s="1" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="36" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1"/>
@@ -3347,7 +3479,7 @@
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
-      <c r="E41" s="13"/>
+      <c r="E41" s="12"/>
       <c r="F41" s="3"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>

</xml_diff>

<commit_message>
correct drifter 6 config file name for deployment 22
</commit_message>
<xml_diff>
--- a/TFO_Drifter_deployment_log.xlsx
+++ b/TFO_Drifter_deployment_log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/sio_research/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2D4E910-04F2-034A-B9A3-49084C93D41F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E3AAB9E-ACAD-6647-AE6D-6D9B90A32833}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38400" yWindow="500" windowWidth="38400" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4529,7 +4529,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R35" s="44" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="S35" s="56">
         <v>45211.82</v>

</xml_diff>

<commit_message>
bug fixes and plot updates
</commit_message>
<xml_diff>
--- a/TFO_Drifter_deployment_log.xlsx
+++ b/TFO_Drifter_deployment_log.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/homes/alaferriere/GIT/sio_research/drifter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/sio_research/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{059C874F-FBB9-2A4F-AC9C-AAF1E119445B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69EC969B-51B8-ED45-9521-512B1517D508}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="500" windowWidth="38400" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="30240" windowHeight="19640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2023" sheetId="1" r:id="rId1"/>
@@ -160,9 +160,6 @@
   </si>
   <si>
     <t>acoustic_config_Drifter6_VS301_2023.txt</t>
-  </si>
-  <si>
-    <t>acoustic_config_Drifter5_VS301_2023.txt</t>
   </si>
   <si>
     <t>Experiment Name</t>
@@ -334,6 +331,9 @@
   </si>
   <si>
     <t>acoustic_config_Drifter5_Acoustic3_VS209_2023.txt</t>
+  </si>
+  <si>
+    <t>acoustic_config_Drifter6_Acoustic4_VS301_2023.txt</t>
   </si>
 </sst>
 </file>
@@ -1663,7 +1663,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="25" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C1" s="25" t="s">
         <v>1</v>
@@ -1678,7 +1678,7 @@
         <v>7</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H1" s="25" t="s">
         <v>8</v>
@@ -1693,7 +1693,7 @@
         <v>17</v>
       </c>
       <c r="L1" s="28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M1" s="25" t="s">
         <v>18</v>
@@ -1732,7 +1732,7 @@
         <v>15</v>
       </c>
       <c r="Y1" s="65" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="Z1" s="31" t="s">
         <v>20</v>
@@ -1741,10 +1741,10 @@
         <v>21</v>
       </c>
       <c r="AB1" s="25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="AC1" s="25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AD1" s="25" t="s">
         <v>22</v>
@@ -1755,7 +1755,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C2" s="32">
         <v>4</v>
@@ -1825,7 +1825,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C3" s="40">
         <v>4</v>
@@ -1910,7 +1910,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C4" s="32">
         <v>4</v>
@@ -1991,7 +1991,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C5" s="40">
         <v>4</v>
@@ -2070,7 +2070,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C6" s="48">
         <v>4</v>
@@ -2151,7 +2151,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C7" s="40">
         <v>4</v>
@@ -2191,7 +2191,7 @@
         <v>300434066482170</v>
       </c>
       <c r="R7" s="44" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S7" s="45">
         <v>44978.792337962965</v>
@@ -2234,7 +2234,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C8" s="48">
         <v>4</v>
@@ -2264,7 +2264,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R8" s="47" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S8" s="52">
         <v>44983.875324074077</v>
@@ -2305,7 +2305,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C9" s="48">
         <v>4</v>
@@ -2335,7 +2335,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R9" s="47" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S9" s="52">
         <v>44984.416990740741</v>
@@ -2376,7 +2376,7 @@
         <v>7</v>
       </c>
       <c r="B10" s="48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C10" s="48">
         <v>4</v>
@@ -2406,7 +2406,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R10" s="47" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S10" s="52">
         <v>44984.896157407406</v>
@@ -2447,7 +2447,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C11" s="48">
         <v>4</v>
@@ -2477,7 +2477,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R11" s="47" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="S11" s="52">
         <v>44985.403113425928</v>
@@ -2518,7 +2518,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C12" s="40">
         <v>5</v>
@@ -2558,7 +2558,7 @@
         <v>300434066482170</v>
       </c>
       <c r="R12" s="44" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="S12" s="45">
         <v>44983.889456018522</v>
@@ -2599,7 +2599,7 @@
         <v>8</v>
       </c>
       <c r="B13" s="48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C13" s="40">
         <v>5</v>
@@ -2629,7 +2629,7 @@
         <v>300434066482170</v>
       </c>
       <c r="R13" s="44" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="S13" s="45">
         <v>44984.410046296296</v>
@@ -2670,7 +2670,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="48" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C14" s="48">
         <v>6</v>
@@ -2747,7 +2747,7 @@
         <v>10</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C15" s="40">
         <v>6</v>
@@ -2832,7 +2832,7 @@
         <v>11</v>
       </c>
       <c r="B16" s="48" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C16" s="48">
         <v>4</v>
@@ -2901,7 +2901,7 @@
         <v>11</v>
       </c>
       <c r="B17" s="48" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C17" s="48">
         <v>4</v>
@@ -2970,7 +2970,7 @@
         <v>12</v>
       </c>
       <c r="B18" s="40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C18" s="40">
         <v>5</v>
@@ -3039,7 +3039,7 @@
         <v>12</v>
       </c>
       <c r="B19" s="40" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C19" s="40">
         <v>5</v>
@@ -3108,7 +3108,7 @@
         <v>13</v>
       </c>
       <c r="B20" s="48" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C20" s="48">
         <v>6</v>
@@ -3122,7 +3122,10 @@
       <c r="F20" s="50">
         <v>0.37708333333333338</v>
       </c>
-      <c r="G20" s="35"/>
+      <c r="G20" s="71">
+        <f t="shared" ref="G20:G35" si="1">$F20+TIME(AC20,0,0)</f>
+        <v>0.66875000000000007</v>
+      </c>
       <c r="H20" s="48">
         <v>32.910367999999998</v>
       </c>
@@ -3132,8 +3135,13 @@
       <c r="J20" s="49">
         <v>45180</v>
       </c>
-      <c r="K20" s="51"/>
-      <c r="L20" s="51"/>
+      <c r="K20" s="51">
+        <v>0.25</v>
+      </c>
+      <c r="L20" s="43">
+        <f>$K20 +TIME($AC20,0,0)</f>
+        <v>0.54166666666666674</v>
+      </c>
       <c r="M20" s="48"/>
       <c r="N20" s="48"/>
       <c r="O20" s="48">
@@ -3146,7 +3154,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R20" s="47" t="s">
-        <v>40</v>
+        <v>97</v>
       </c>
       <c r="S20" s="54">
         <v>45176.681122685186</v>
@@ -3176,8 +3184,12 @@
       <c r="AA20" s="53">
         <v>6.2847222222222221E-2</v>
       </c>
-      <c r="AB20" s="48"/>
-      <c r="AC20" s="48"/>
+      <c r="AB20" s="48">
+        <v>250</v>
+      </c>
+      <c r="AC20" s="48">
+        <v>7</v>
+      </c>
       <c r="AD20" s="48"/>
     </row>
     <row r="21" spans="1:30" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3185,7 +3197,7 @@
         <v>14</v>
       </c>
       <c r="B21" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C21" s="40">
         <v>4</v>
@@ -3200,7 +3212,7 @@
         <v>0.29722222222222222</v>
       </c>
       <c r="G21" s="71">
-        <f t="shared" ref="G21:G35" si="1">$F21+TIME(AC21,0,0)</f>
+        <f t="shared" si="1"/>
         <v>0.46388888888888891</v>
       </c>
       <c r="H21" s="40">
@@ -3235,7 +3247,7 @@
         <v>300434066489180</v>
       </c>
       <c r="R21" s="44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S21" s="45">
         <v>45203.501250000001</v>
@@ -3272,7 +3284,7 @@
         <v>4</v>
       </c>
       <c r="AD21" s="40" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:30" s="23" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3280,7 +3292,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="48" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C22" s="48">
         <v>5</v>
@@ -3367,7 +3379,7 @@
         <v>4</v>
       </c>
       <c r="AD22" s="48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" spans="1:30" s="23" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3375,7 +3387,7 @@
         <v>15</v>
       </c>
       <c r="B23" s="48" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23" s="48">
         <v>5</v>
@@ -3462,7 +3474,7 @@
         <v>4</v>
       </c>
       <c r="AD23" s="48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:30" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3470,7 +3482,7 @@
         <v>16</v>
       </c>
       <c r="B24" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C24" s="40">
         <v>6</v>
@@ -3520,7 +3532,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R24" s="44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S24" s="56">
         <v>45203.528344907405</v>
@@ -3563,7 +3575,7 @@
         <v>16</v>
       </c>
       <c r="B25" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C25" s="40">
         <v>6</v>
@@ -3613,7 +3625,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R25" s="44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S25" s="56">
         <v>45204.771168981482</v>
@@ -3656,7 +3668,7 @@
         <v>17</v>
       </c>
       <c r="B26" s="48" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C26" s="48">
         <v>6</v>
@@ -3706,7 +3718,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R26" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S26" s="54">
         <v>45208.132511574076</v>
@@ -3749,7 +3761,7 @@
         <v>17</v>
       </c>
       <c r="B27" s="48" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C27" s="48">
         <v>6</v>
@@ -3799,7 +3811,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R27" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S27" s="54">
         <v>45208.771828703706</v>
@@ -3842,7 +3854,7 @@
         <v>17</v>
       </c>
       <c r="B28" s="48" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C28" s="48">
         <v>6</v>
@@ -3892,7 +3904,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R28" s="47" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S28" s="54">
         <v>45209.750567129631</v>
@@ -3935,7 +3947,7 @@
         <v>18</v>
       </c>
       <c r="B29" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C29" s="40">
         <v>4</v>
@@ -3985,7 +3997,7 @@
         <v>300434066489180</v>
       </c>
       <c r="R29" s="44" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S29" s="56">
         <v>45208.1325</v>
@@ -4022,7 +4034,7 @@
         <v>4</v>
       </c>
       <c r="AD29" s="40" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30" spans="1:30" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4030,7 +4042,7 @@
         <v>18</v>
       </c>
       <c r="B30" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C30" s="40">
         <v>4</v>
@@ -4080,7 +4092,7 @@
         <v>300434066489180</v>
       </c>
       <c r="R30" s="44" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="S30" s="56">
         <v>45208.764548611114</v>
@@ -4123,7 +4135,7 @@
         <v>19</v>
       </c>
       <c r="B31" s="48" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C31" s="48">
         <v>5</v>
@@ -4210,7 +4222,7 @@
         <v>4</v>
       </c>
       <c r="AD31" s="48" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:30" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4218,7 +4230,7 @@
         <v>20</v>
       </c>
       <c r="B32" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C32" s="40">
         <v>5</v>
@@ -4305,7 +4317,7 @@
         <v>4</v>
       </c>
       <c r="AD32" s="40" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="1:30" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4313,7 +4325,7 @@
         <v>20</v>
       </c>
       <c r="B33" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C33" s="40">
         <v>5</v>
@@ -4406,7 +4418,7 @@
         <v>21</v>
       </c>
       <c r="B34" s="48" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C34" s="48">
         <v>4</v>
@@ -4456,7 +4468,7 @@
         <v>300434066489180</v>
       </c>
       <c r="R34" s="47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S34" s="54">
         <v>45211.834328703706</v>
@@ -4493,7 +4505,7 @@
         <v>4</v>
       </c>
       <c r="AD34" s="48" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:30" s="24" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4501,7 +4513,7 @@
         <v>22</v>
       </c>
       <c r="B35" s="40" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C35" s="40">
         <v>6</v>
@@ -4551,7 +4563,7 @@
         <v>300434066480130</v>
       </c>
       <c r="R35" s="44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="S35" s="56">
         <v>45211.82</v>
@@ -4588,7 +4600,7 @@
         <v>4</v>
       </c>
       <c r="AD35" s="40" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -35628,100 +35640,100 @@
   <sheetData>
     <row r="1" spans="1:34" ht="96" x14ac:dyDescent="0.2">
       <c r="A1" s="72" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B1" s="73"/>
       <c r="C1" s="73"/>
       <c r="D1" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E1" s="22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F1" s="22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G1" s="22" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H1" s="22"/>
       <c r="I1" s="22" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J1" s="22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K1" s="22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="L1" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="M1" s="22" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="N1" s="22" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="O1" s="22" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P1" s="22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="Q1" s="22" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="R1" s="22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="S1" s="22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="T1" s="22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="U1" s="22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="V1" s="22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="W1" s="22" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="X1" s="22" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="Y1" s="22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="Z1" s="22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="AA1" s="22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="AB1" s="22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="AC1" s="22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AD1" s="22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AE1" s="22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AF1" s="22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AG1" s="22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="AH1" s="22" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.2">
@@ -35850,7 +35862,7 @@
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B3" s="21">
         <v>38.826842999999997</v>
@@ -35978,7 +35990,7 @@
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B4" s="21">
         <v>-63.845635000000001</v>
@@ -35993,7 +36005,7 @@
     </row>
     <row r="5" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A5" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B5" s="20">
         <v>0</v>
@@ -36017,7 +36029,7 @@
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A7" s="14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7" s="19">
         <v>45204</v>

</xml_diff>

<commit_message>
updating log file as run on macmussel
</commit_message>
<xml_diff>
--- a/TFO_Drifter_deployment_log.xlsx
+++ b/TFO_Drifter_deployment_log.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alaferri/GIT/sio_code/sio_research_merge/drifter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/homes/alaferriere/GIT/sio_research/drifter/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C66609BD-EEB8-A440-A1E4-3749D947C988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1D84052-5AB9-0244-A77D-E7BF8B2EC36A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10340" yWindow="3600" windowWidth="38400" windowHeight="19960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Drifter Log 2022-2023" sheetId="1" r:id="rId1"/>
@@ -501,7 +501,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="167" fontId="9" fillId="0" borderId="0" xfId="2" applyNumberFormat="1"/>
@@ -671,6 +671,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="20% - Accent3" xfId="1" builtinId="38"/>
@@ -1953,7 +1954,7 @@
         <v>-63.696891999999998</v>
       </c>
       <c r="Y4" s="52">
-        <f t="shared" ref="Y4:Y35" si="0">(V4-S4)*1440/60</f>
+        <f t="shared" ref="Y4:Y38" si="0">(V4-S4)*1440/60</f>
         <v>9.1666666666860692</v>
       </c>
       <c r="Z4" s="24">
@@ -4661,9 +4662,16 @@
       <c r="X36" s="25">
         <v>-117.66408699999999</v>
       </c>
-      <c r="Y36" s="52"/>
-      <c r="Z36" s="31"/>
-      <c r="AA36" s="31"/>
+      <c r="Y36" s="52">
+        <f t="shared" si="0"/>
+        <v>24.083333333255723</v>
+      </c>
+      <c r="Z36" s="31">
+        <v>0.6166666666666667</v>
+      </c>
+      <c r="AA36" s="31">
+        <v>5.2777777777777778E-2</v>
+      </c>
       <c r="AB36" s="25"/>
       <c r="AC36" s="25">
         <v>8</v>
@@ -4737,9 +4745,16 @@
       <c r="X37" s="25">
         <v>-117.6035</v>
       </c>
-      <c r="Y37" s="52"/>
-      <c r="Z37" s="31"/>
-      <c r="AA37" s="31"/>
+      <c r="Y37" s="52">
+        <f t="shared" si="0"/>
+        <v>22.744166666641831</v>
+      </c>
+      <c r="Z37" s="31">
+        <v>0.6166666666666667</v>
+      </c>
+      <c r="AA37" s="31">
+        <v>5.2777777777777778E-2</v>
+      </c>
       <c r="AB37" s="25"/>
       <c r="AC37" s="25">
         <v>8</v>
@@ -4795,15 +4810,34 @@
       <c r="R38" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="S38" s="30"/>
-      <c r="T38" s="25"/>
-      <c r="U38" s="25"/>
-      <c r="V38" s="30"/>
-      <c r="W38" s="25"/>
-      <c r="X38" s="25"/>
-      <c r="Y38" s="52"/>
-      <c r="Z38" s="31"/>
-      <c r="AA38" s="31"/>
+      <c r="S38" s="30">
+        <v>45317.875324074077</v>
+      </c>
+      <c r="T38" s="63">
+        <v>32.909129</v>
+      </c>
+      <c r="U38" s="63">
+        <v>-117.680663</v>
+      </c>
+      <c r="V38" s="30">
+        <v>45318.878796296296</v>
+      </c>
+      <c r="W38" s="63">
+        <v>32.999972</v>
+      </c>
+      <c r="X38" s="63">
+        <v>-117.66408699999999</v>
+      </c>
+      <c r="Y38" s="52">
+        <f t="shared" si="0"/>
+        <v>24.083333333255723</v>
+      </c>
+      <c r="Z38" s="31">
+        <v>0.6166666666666667</v>
+      </c>
+      <c r="AA38" s="31">
+        <v>5.2777777777777778E-2</v>
+      </c>
       <c r="AB38" s="25"/>
       <c r="AC38" s="25">
         <v>8</v>

</xml_diff>